<commit_message>
feat: upgrade optimization engine to v3 with best-fit board matching and rotation support
</commit_message>
<xml_diff>
--- a/data/t1_inventory.xlsx
+++ b/data/t1_inventory.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,26 +413,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>board_type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Height</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Depth</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty</t>
         </is>
@@ -453,32 +441,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T1-610*2440</t>
+          <t>T0-1219.2x2438.4</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2440</v>
+        <v>2438.4</v>
       </c>
       <c r="C2" t="n">
-        <v>285.8</v>
+        <v>1219.2</v>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T1-1220*2440</t>
+          <t>T1-304.8x2438.4</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2440</v>
+        <v>2438.4</v>
       </c>
       <c r="C3" t="n">
-        <v>590.6</v>
+        <v>304.8</v>
       </c>
       <c r="D3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T1-609.6x2438.4</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2438.4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>609.6</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T1-286.8x2438.4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2438.4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>286.8</v>
+      </c>
+      <c r="D5" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: remove legacy API server and workflows while enhancing cloud controller error handling and project structure
</commit_message>
<xml_diff>
--- a/data/t1_inventory.xlsx
+++ b/data/t1_inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,7 +429,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Depth</t>
+          <t>Width</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -499,6 +499,22 @@
         <v>286.8</v>
       </c>
       <c r="D5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T1-101.6x2438.4</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2438.4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="D6" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>